<commit_message>
Khởi tạo dự án, thiết kế Database, xây dựng kế hoạch dự án
</commit_message>
<xml_diff>
--- a/Phan_Cong.xlsx
+++ b/Phan_Cong.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SCHOOL\Hk2_nam_3\Quan_Tri_Du_An_CNTT\btth9\NguyenTuanAnh\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4AF2E6-2C4A-4F5A-8099-F8741B6F6FE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CDB1019-061D-4987-9E0F-08DB7EF1E18A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{38B4B71A-B216-4752-AB30-749D8880233C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{38B4B71A-B216-4752-AB30-749D8880233C}"/>
   </bookViews>
   <sheets>
     <sheet name="Bang_Thanh_Vien" sheetId="1" r:id="rId1"/>
-    <sheet name="Bang_Cong_Viec" sheetId="2" r:id="rId2"/>
+    <sheet name="Gioi_thieu_Du_An" sheetId="2" r:id="rId2"/>
+    <sheet name="Phan_Cong" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
   <si>
     <t>Danh sách thành viên tham gia làm dự án</t>
   </si>
@@ -66,17 +67,170 @@
     <t>Thành viên</t>
   </si>
   <si>
-    <t xml:space="preserve">Danh sách công việc </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
+    <t>Tên dự án</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Công nghệ sử dụng </t>
+  </si>
+  <si>
+    <t>Mục đích</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mục tiêu </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Hệ thống quản trị dự án CNTT</t>
+  </si>
+  <si>
+    <t>ReactJS + FastAPI + PostgreSQL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xây dựng hệ thống website quản lý CNTT giúp các đội nhóm dự án dễ dàng lập kế hoạch, theo dõi tiến độ, kiểm tra chặt chẽ thời gian, chi phí một cách hiệu quả. </t>
+  </si>
+  <si>
+    <t>Hoàn thành thiết kế, lập trình và triển khai dự án ổn định.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hỗ trợ phân quyền Trưởng dự án và Đội dự án. Quản lý truy cập thông qua mã dự án. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoàn thiện các chức năng cốt lõi: </t>
+  </si>
+  <si>
+    <t>1.Quản lý công việc</t>
+  </si>
+  <si>
+    <t>2.Ước lượng thời gian công việc (Expert)</t>
+  </si>
+  <si>
+    <t>3.Ước lượng chi phí cho dự án</t>
+  </si>
+  <si>
+    <t>4.Quản lý lịch trình dự án</t>
+  </si>
+  <si>
+    <t>5.Quản lý lịch trình công việc cho dự án</t>
+  </si>
+  <si>
+    <t>Nộp đẩy đủ tài liệu (Source code cập nhật theo buổi, file phân công nhiệm vụ, file những việc đã làm trong buổi thực hành)</t>
+  </si>
+  <si>
+    <t>Mã CV</t>
+  </si>
+  <si>
+    <t>Khởi tạo &amp; Phân quyền (Login)</t>
+  </si>
+  <si>
+    <t>Setup base project</t>
+  </si>
+  <si>
+    <t>Tạo dự án Vite + React + Tailwind</t>
+  </si>
+  <si>
+    <t>Khởi tạo FastAPI + SQLAlchemy</t>
+  </si>
+  <si>
+    <t>Thiết kế Database</t>
+  </si>
+  <si>
+    <t>(Phối hợp chốt schema JSON)</t>
+  </si>
+  <si>
+    <t>Thiết kế 4 bảng (Users, Projects, Tasks...)</t>
+  </si>
+  <si>
+    <t>Chức năng Đăng nhập &amp; Auth</t>
+  </si>
+  <si>
+    <t>Dựng Form Login, lưu Token (Local Storage)</t>
+  </si>
+  <si>
+    <t>Code API Login, tạo &amp; mã hóa JWT</t>
+  </si>
+  <si>
+    <t>Join dự án bằng Mã (Project Code)</t>
+  </si>
+  <si>
+    <t>Dựng Form nhập mã, gọi API join dự án</t>
+  </si>
+  <si>
+    <t>Code API kiểm tra mã &amp; phân quyền</t>
+  </si>
+  <si>
+    <t>Giao diện Bảng công việc (WBS)</t>
+  </si>
+  <si>
+    <t>Dùng AntD/MUI dựng Table hiển thị dạng Cha-Con</t>
+  </si>
+  <si>
+    <t>API CRUD (Thêm/Sửa/Xóa/Lấy) cho bảng Tasks</t>
+  </si>
+  <si>
+    <t>Tính toán PERT (Thời gian)</t>
+  </si>
+  <si>
+    <t>Làm Form nhập 3 số MO, ML, MP</t>
+  </si>
+  <si>
+    <t>Viết logic tính EST, cập nhật vào DB</t>
+  </si>
+  <si>
+    <t>Quản lý Chi phí</t>
+  </si>
+  <si>
+    <t>Thêm cột nhập Tiền vào bảng Table</t>
+  </si>
+  <si>
+    <t>Cập nhật API Tasks để nhận &amp; lưu biến số Tiền</t>
+  </si>
+  <si>
+    <t>Trực quan hóa (Kanban &amp; Gantt)</t>
+  </si>
+  <si>
+    <t>Bảng Kanban (Kéo thả thẻ)</t>
+  </si>
+  <si>
+    <t>Tích hợp thư viện (dnd-kit), code giao diện kéo thả</t>
+  </si>
+  <si>
+    <t>API Update Status (/tasks/{id}/status)</t>
+  </si>
+  <si>
+    <t>Biểu đồ Gantt</t>
+  </si>
+  <si>
+    <t>Tích hợp thư viện Gantt, map data ngày tháng</t>
+  </si>
+  <si>
+    <t>(Đã có data từ API Tasks, hỗ trợ test)</t>
+  </si>
+  <si>
+    <t>Tổng duyệt &amp; Báo cáo</t>
+  </si>
+  <si>
+    <t>Viết file báo cáo UI/UX, hướng dẫn sử dụng</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Frontend (Tuấn Anh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Backend (Vũ)</t>
+  </si>
+  <si>
+    <t>Hạng mục công việc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quản lý WBS &amp; PERT </t>
+  </si>
+  <si>
+    <t>Khởi chạy test Postman hoặc Swagger UI, fix bug logic API</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,6 +260,56 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -127,7 +331,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -264,14 +468,142 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -281,38 +613,87 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -657,53 +1038,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="5"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="16"/>
       <c r="E1" s="2"/>
     </row>
     <row r="2" spans="1:5" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="21" x14ac:dyDescent="0.4">
-      <c r="A3" s="9">
+      <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="7">
         <v>23050118</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="9" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="13">
+      <c r="A4" s="10">
         <v>2</v>
       </c>
-      <c r="B4" s="14">
+      <c r="B4" s="11">
         <v>23050102</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="13" t="s">
         <v>8</v>
       </c>
     </row>
@@ -723,18 +1104,416 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE9D5286-D0A4-4B83-83AE-C4FC632A9FE3}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:S12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.21875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:19" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+    </row>
+    <row r="2" spans="1:19" ht="36" x14ac:dyDescent="0.35">
+      <c r="A2" s="19" t="s">
         <v>10</v>
       </c>
+      <c r="B2" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+    </row>
+    <row r="3" spans="1:19" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="18"/>
+      <c r="S3" s="18"/>
+    </row>
+    <row r="4" spans="1:19" ht="18" x14ac:dyDescent="0.35">
+      <c r="A4" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+    </row>
+    <row r="5" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="26"/>
+      <c r="B5" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+    </row>
+    <row r="6" spans="1:19" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="26"/>
+      <c r="B6" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+    </row>
+    <row r="7" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="26"/>
+      <c r="B7" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+    </row>
+    <row r="8" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="26"/>
+      <c r="B8" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+    </row>
+    <row r="9" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="26"/>
+      <c r="B9" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+    </row>
+    <row r="10" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="26"/>
+      <c r="B10" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+    </row>
+    <row r="11" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="26"/>
+      <c r="B11" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+    </row>
+    <row r="12" spans="1:19" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="27"/>
+      <c r="B12" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
     </row>
   </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="A4:A12"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B2:G2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D631DB77-8D3F-4640-BBBB-D5BF95C6B06C}">
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.88671875" customWidth="1"/>
+    <col min="2" max="2" width="44.44140625" customWidth="1"/>
+    <col min="3" max="3" width="48.6640625" customWidth="1"/>
+    <col min="4" max="4" width="45.21875" customWidth="1"/>
+    <col min="5" max="5" width="27.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="31.2" x14ac:dyDescent="0.6">
+      <c r="A1" s="30" t="str">
+        <f>UPPER("Danh sách công việc cần lầm")</f>
+        <v>DANH SÁCH CÔNG VIỆC CẦN LẦM</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="32"/>
+    </row>
+    <row r="2" spans="1:5" ht="39.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="38" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="39" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="39" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="39" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" s="40" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="41">
+        <v>1</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="44"/>
+    </row>
+    <row r="4" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="34">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="33"/>
+    </row>
+    <row r="5" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="34">
+        <v>1.2</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="33"/>
+    </row>
+    <row r="6" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="34">
+        <v>1.3</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="33"/>
+    </row>
+    <row r="7" spans="1:5" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="35">
+        <v>1.4</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="37"/>
+    </row>
+    <row r="8" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="41">
+        <v>2</v>
+      </c>
+      <c r="B8" s="42" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="44"/>
+    </row>
+    <row r="9" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="34">
+        <v>2.1</v>
+      </c>
+      <c r="B9" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="33"/>
+    </row>
+    <row r="10" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="34">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="33"/>
+    </row>
+    <row r="11" spans="1:5" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="35">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="B11" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="36" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="36" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="37"/>
+    </row>
+    <row r="12" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="41">
+        <v>3</v>
+      </c>
+      <c r="B12" s="42" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="44"/>
+    </row>
+    <row r="13" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="34">
+        <v>3.1</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="E13" s="33"/>
+    </row>
+    <row r="14" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="34">
+        <v>3.2</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="33"/>
+    </row>
+    <row r="15" spans="1:5" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="35">
+        <v>3.3</v>
+      </c>
+      <c r="B15" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="36" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="37"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="17"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="17"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>